<commit_message>
april panic and paper progress
</commit_message>
<xml_diff>
--- a/PowerAnalysis.xlsx
+++ b/PowerAnalysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33ab2cc4ec646a75/Documents/GitHub/Treadmill/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{033314CD-06CF-40D5-B58D-2B4B3135AA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{817F4F4C-8A5B-4790-BB7A-56B44440D307}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{033314CD-06CF-40D5-B58D-2B4B3135AA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D47DA3C1-396E-4382-8779-39245AE6D17E}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{DB461667-9DE4-470E-A3E5-C407E91C9246}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{DB461667-9DE4-470E-A3E5-C407E91C9246}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>power analysis for split-belt treadmill</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>Stenum and choi</t>
+  </si>
+  <si>
+    <t>retention paper</t>
   </si>
 </sst>
 </file>
@@ -565,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9E018C4-79F3-4BDF-B230-C4603E087834}">
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" style="1" customWidth="1"/>
@@ -905,6 +908,9 @@
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>47</v>
+      </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -920,10 +926,7 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>44</v>
-      </c>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -939,7 +942,10 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1017,6 +1023,7 @@
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
@@ -1075,6 +1082,8 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
@@ -1141,6 +1150,19 @@
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
     </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>